<commit_message>
Update path in publication-request.json ee2001dd0d56665e5579f2091c0c7570b4111dbe
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-dmi-classe-risque.xlsx
+++ b/main/ig/StructureDefinition-dmi-classe-risque.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-05T10:01:25+00:00</t>
+    <t>2026-03-05T10:22:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1106,7 +1106,7 @@
         <v>78</v>
       </c>
       <c r="AI4" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ4" t="s" s="2">
         <v>81</v>
@@ -1314,7 +1314,7 @@
         <v>83</v>
       </c>
       <c r="AI6" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ6" t="s" s="2">
         <v>106</v>

</xml_diff>